<commit_message>
render conference presentations and other publications automatically from XLSX file
</commit_message>
<xml_diff>
--- a/_outputs.xlsx
+++ b/_outputs.xlsx
@@ -5,10 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="articles" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="conferences" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="other" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="128">
   <si>
     <t xml:space="preserve">authors</t>
   </si>
@@ -339,6 +341,72 @@
   <si>
     <t xml:space="preserve">16 June 2022</t>
   </si>
+  <si>
+    <t xml:space="preserve">conference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACR Convergence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Washington, D.C.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">November 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost-effectiveness of low dose colchicine prophylaxis when starting allopurinol using the "Start-Low Go-Slow" approach for gout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">poster presentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OARSI World Congress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vienna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">April 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Health system and societal costs following osteoarthritis diagnosis in primary care</t>
+  </si>
+  <si>
+    <t xml:space="preserve">with</t>
+  </si>
+  <si>
+    <t xml:space="preserve">available</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistical Analysis Plan for Reducing the burden of knee osteoarthritis through community pharmacy: A randomised controlled trial of the Knee Care for Arthritis through Pharmacy Service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">James Stanley and Ben Darlow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 October 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://hdl.handle.net/10523/42913</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Economic evaluation of the effects of manual therapy for knee osteoarthritis: Study protocol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yana Pryymachenko, Haxby Abbott, and Cathy Chapple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 May 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://osf.io/arn9v/</t>
+  </si>
 </sst>
 </file>
 
@@ -429,7 +497,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -456,6 +524,10 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -17399,4 +17471,149 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="7" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="101.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="43.26"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="7" width="15.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="28.52"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="7" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add GRoC validity paper to publications
</commit_message>
<xml_diff>
--- a/_outputs.xlsx
+++ b/_outputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilro23p\Documents\rosswilson-nz.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7AE12AD-1411-41C9-98E6-55A7D0EF3D49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A45A11-D672-4119-BFCA-64A8785FC944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="481">
   <si>
     <t>authors</t>
   </si>
@@ -1476,6 +1476,24 @@
   </si>
   <si>
     <t>**Background**&lt;br&gt;Multimorbidity – the co-existence of two or more chronic health conditions in the same individual, without reference to an index condition – has become a global health issue and creates enormous pressure on the healthcare system. This review aimed to summarise evidence on the effectiveness of interventions used to manage people with multimorbidity.&lt;br&gt;&lt;br&gt;**Methods**&lt;br&gt;MEDLINE, EMBASE, CINAHL, Cochrane Library, two trials registers, and grey literature were searched for studies of adults with multimorbidity receiving care in primary or community care settings up to 30-September-2024. Two reviewers independently screened studies for eligibility, extracted data, and assessed risk of bias and study certainty. Interventions were categorised as medicines management (MM), support for self-management (SSM), or care coordination plus support for self-management (CC+SSM). Meta-analyses for primary outcomes (health-related quality of life, healthcare utilisation, and healthcare costs) were conducted.&lt;br&gt;&lt;br&gt;**Results**&lt;br&gt;From 10,272 titles screened, 33 eligible studies (this review:18, previous review:15; MM:6, SSM:9, CC+SSM:18) were identified, of which 26 studies with 9,449 participants were included in meta-analysis. Overall, there was little significant evidence of benefit of the interventions compared to usual care for most outcomes. SSM was associated with lower hospitalisation risk and medication costs, but slightly more emergency department (ED) visits; and CC+SSM with better SF-12 PCS score, lower hospitalisation risk and fewer ED visits, but more outpatient and general practitioner visits.&lt;br&gt;&lt;br&gt;**Conclusion**&lt;br&gt;This review found some suggestions of improved outcomes and reduced healthcare utilisation (especially hospitalisation) for these interventions. There is a paucity of evidence reporting on health outcomes, especially healthcare costs, in the management of multimorbidity.</t>
+  </si>
+  <si>
+    <t>Pierobon A. Gaspar Fernandes L, Wilson R, Christopherson RM, Stanley J, Pryymachenko Y, Lim YW, Caya R, Gayed M, Abbott H</t>
+  </si>
+  <si>
+    <t>Validity of the Global Rating of Change in patients with chronic low back pain</t>
+  </si>
+  <si>
+    <t>10.1016/j.msksp.2025.103443</t>
+  </si>
+  <si>
+    <t>8 November 2025</t>
+  </si>
+  <si>
+    <t>**Background**&lt;br&gt;The Global Rating of Change (GROC) is a widely used outcome measure that aims to capture change in overall health status. There is limited evidence on the validity of the GROC for measuring change among patients with chronic low back pain (CLBP), and little is known about which clinical variables explain the GROC score.&lt;br&gt;&lt;br&gt;**Objectives**&lt;br&gt;This study aimed to assess the validity of the GROC in measuring change, and identify which clinical variables correlate with the GROC score in patients with CLBP.&lt;br&gt;&lt;br&gt;**Design**&lt;br&gt;Retrospective observational study.&lt;br&gt;&lt;br&gt;**Methods**&lt;br&gt;This secondary analysis included clinical data from patients with CLBP enrolled in a physiotherapy program. Data on pain intensity, function, pain catastrophizing, depression, and quality of life were collected at baseline and discharge, and the GROC scale was completed at discharge. We performed Spearman correlation and linear regression analyses to examine the relationship between the GROC and change/discharge scores for all clinical variables.&lt;br&gt;&lt;br&gt;**Results**&lt;br&gt;Data from 102 participants were analysed. Spearman correlations between the GROC and discharge scores were greater (-0.46 to -0.71) than correlations between the GROC and change scores (-0.34 to -0.63) for all variables. The linear regression model including discharge scores explained a greater part of the variance of the GROC score (R&lt;sup&gt;2&lt;/sup&gt; = 0.63) than the model including change scores (R&lt;sup&gt;2&lt;/sup&gt; = 0.46). In both models, pain intensity was the variable most strongly associated with the GROC score.&lt;br&gt;&lt;br&gt;**Conclusion**&lt;br&gt;Baseline and discharge outcome measures should be preferred over the GROC for measuring change after treatment in patients with CLBP.</t>
+  </si>
+  <si>
+    <t>Musculoskeletal Science and Practice</t>
   </si>
 </sst>
 </file>
@@ -1715,7 +1733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="1"/>
@@ -1763,15 +1781,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="242.25" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>20</v>
+        <v>480</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>13</v>
@@ -1779,22 +1797,25 @@
       <c r="G2" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="H2" s="1" t="s">
+        <v>477</v>
+      </c>
       <c r="I2" s="1" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>12</v>
+        <v>478</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="242.25" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>13</v>
@@ -1802,545 +1823,536 @@
       <c r="G3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+    <row r="5" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D5" s="1">
         <v>41</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E5" s="1">
         <v>6</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G5" s="1">
         <v>2024</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="255" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+    <row r="6" spans="1:10" ht="255" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="280.5" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>30</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="89.25" x14ac:dyDescent="0.2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="280.5" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>30</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>50</v>
+        <v>40</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="242.25" x14ac:dyDescent="0.2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="89.25" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>30</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>59</v>
+        <v>49</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>50</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="242.25" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>64</v>
+        <v>55</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>56</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>30</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>12</v>
+        <v>63</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>30</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>79</v>
+        <v>12</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>55</v>
+        <v>71</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>30</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="293.25" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>30</v>
       </c>
       <c r="H12" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="293.25" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="165.75" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+    <row r="14" spans="1:10" ht="165.75" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C14" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="267.75" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>94</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>96</v>
       </c>
       <c r="H14" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="267.75" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="I15" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="280.5" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
+    <row r="16" spans="1:10" ht="280.5" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B16" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D16" s="6">
         <v>52</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E16" s="6">
         <v>5</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="G15" s="6">
+      <c r="G16" s="6">
         <v>2022</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H16" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="I16" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="J15" s="6" t="s">
+      <c r="J16" s="6" t="s">
         <v>112</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
-      <c r="A16" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="H16" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
+      <c r="A18" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B18" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C18" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D18" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>134</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>126</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="293.25" x14ac:dyDescent="0.2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>71</v>
+        <v>37</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>133</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>126</v>
       </c>
       <c r="H19" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="293.25" x14ac:dyDescent="0.2">
+      <c r="A20" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="H20" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="I20" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="J19" s="1" t="s">
+      <c r="J20" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
-      <c r="A20" s="8" t="s">
+    <row r="21" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
+      <c r="A21" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B21" s="8" t="s">
         <v>146</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="H20" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="242.25" x14ac:dyDescent="0.2">
-      <c r="A21" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>154</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>147</v>
@@ -2352,59 +2364,59 @@
         <v>56</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>149</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="204" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" ht="242.25" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>160</v>
+        <v>38</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>161</v>
+        <v>56</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>149</v>
       </c>
       <c r="H22" s="10" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="153" x14ac:dyDescent="0.2">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="204" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>132</v>
@@ -2413,245 +2425,248 @@
         <v>160</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>149</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="191.25" x14ac:dyDescent="0.2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="153" x14ac:dyDescent="0.2">
       <c r="A24" s="8" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>175</v>
+        <v>132</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>133</v>
+        <v>160</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>47</v>
+        <v>168</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>149</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="191.25" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>160</v>
+        <v>133</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>182</v>
+        <v>47</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>149</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="153" x14ac:dyDescent="0.2">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A26" s="8" t="s">
-        <v>187</v>
+        <v>166</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>190</v>
+        <v>160</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>182</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>149</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="191.25" x14ac:dyDescent="0.2">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="153" x14ac:dyDescent="0.2">
       <c r="A27" s="8" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="G27" s="1" t="s">
         <v>149</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="191.25" x14ac:dyDescent="0.2">
       <c r="A28" s="8" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>132</v>
+        <v>197</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>160</v>
+        <v>198</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>133</v>
+        <v>182</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="G28" s="1" t="s">
         <v>149</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="102" x14ac:dyDescent="0.2">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="191.25" x14ac:dyDescent="0.2">
       <c r="A29" s="8" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>211</v>
+        <v>132</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>212</v>
+        <v>160</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>213</v>
+        <v>133</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>149</v>
       </c>
+      <c r="H29" s="10" t="s">
+        <v>206</v>
+      </c>
       <c r="I29" s="1" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="J29" s="1" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="165.75" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" ht="102" x14ac:dyDescent="0.2">
       <c r="A30" s="8" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>222</v>
+        <v>149</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>224</v>
+        <v>208</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="165.75" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="C31" s="9" t="s">
         <v>218</v>
@@ -2660,398 +2675,427 @@
         <v>219</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="G31" s="1" t="s">
         <v>222</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="409.5" x14ac:dyDescent="0.2">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="165.75" x14ac:dyDescent="0.2">
       <c r="A32" s="8" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>182</v>
+        <v>227</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="H32" s="10" t="s">
-        <v>236</v>
-      </c>
       <c r="I32" s="1" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="242.25" x14ac:dyDescent="0.2">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A33" s="8" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>47</v>
+        <v>182</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="G33" s="1" t="s">
         <v>222</v>
       </c>
       <c r="H33" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="242.25" x14ac:dyDescent="0.2">
+      <c r="A34" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="H34" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="I33" s="1" t="s">
+      <c r="I34" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="J33" s="1" t="s">
+      <c r="J34" s="1" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="178.5" x14ac:dyDescent="0.2">
-      <c r="A34" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="C34" s="9" t="s">
-        <v>248</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="H34" s="10" t="s">
-        <v>252</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" ht="178.5" x14ac:dyDescent="0.2">
       <c r="A35" s="8" t="s">
         <v>225</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>56</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>251</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A36" s="8" t="s">
-        <v>261</v>
+        <v>225</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>263</v>
+        <v>241</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>251</v>
       </c>
       <c r="H36" s="10" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A37" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>266</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
+      <c r="A38" s="8" t="s">
         <v>269</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="B38" s="8" t="s">
         <v>270</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C38" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D38" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="E38" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="F38" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="G38" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="H37" s="10" t="s">
+      <c r="H38" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="I38" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="J37" s="1" t="s">
+      <c r="J38" s="1" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="255" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="s">
+    <row r="39" spans="1:10" ht="255" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B39" s="8" t="s">
         <v>278</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="C39" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D39" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="F39" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="G38" s="1" t="s">
+      <c r="G39" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="H38" s="10" t="s">
+      <c r="H39" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="I38" s="1" t="s">
+      <c r="I39" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="J38" s="1" t="s">
+      <c r="J39" s="1" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="267.75" x14ac:dyDescent="0.2">
-      <c r="A39" s="8" t="s">
+    <row r="40" spans="1:10" ht="267.75" x14ac:dyDescent="0.2">
+      <c r="A40" s="8" t="s">
         <v>286</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="B40" s="8" t="s">
         <v>287</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="C40" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D40" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="F40" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G39" s="1" t="s">
+      <c r="G40" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="H39" s="10" t="s">
+      <c r="H40" s="10" t="s">
         <v>290</v>
       </c>
-      <c r="I39" s="1" t="s">
+      <c r="I40" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="J39" s="1" t="s">
+      <c r="J40" s="1" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
-      <c r="A40" s="8" t="s">
+    <row r="41" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
+      <c r="A41" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B41" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="C41" s="9" t="s">
         <v>295</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D41" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="F41" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="G41" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="H40" s="10" t="s">
+      <c r="H41" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="I40" s="1" t="s">
+      <c r="I41" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="J40" s="1" t="s">
+      <c r="J41" s="1" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="382.5" x14ac:dyDescent="0.2">
-      <c r="A41" s="8" t="s">
+    <row r="42" spans="1:10" ht="382.5" x14ac:dyDescent="0.2">
+      <c r="A42" s="8" t="s">
         <v>302</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B42" s="8" t="s">
         <v>303</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C42" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="E42" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="F42" s="1" t="s">
         <v>305</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="H41" s="10" t="s">
-        <v>307</v>
-      </c>
-      <c r="I41" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="165.75" x14ac:dyDescent="0.2">
-      <c r="A42" s="8" t="s">
-        <v>310</v>
-      </c>
-      <c r="B42" s="8" t="s">
-        <v>311</v>
-      </c>
-      <c r="C42" s="9" t="s">
-        <v>288</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>312</v>
       </c>
       <c r="G42" s="1" t="s">
         <v>306</v>
       </c>
       <c r="H42" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="165.75" x14ac:dyDescent="0.2">
+      <c r="A43" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>311</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="H43" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="I42" s="1" t="s">
+      <c r="I43" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="J42" s="1" t="s">
+      <c r="J43" s="1" t="s">
         <v>315</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="H6" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="H7" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="H8" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="H9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="H10" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="H11" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="H12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="H13" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="H14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="H15" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="H16" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="H17" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="H18" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="H19" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="H20" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="H21" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="H22" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="H23" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="H24" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="H25" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="H26" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="H27" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="H28" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="H32" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="H33" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="H34" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="H35" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="H36" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="H37" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="H38" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="H39" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="H40" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="H41" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="H42" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="H6" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="H7" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="H8" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="H9" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="H10" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="H11" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="H12" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="H13" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="H14" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="H15" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="H16" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="H17" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="H18" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="H19" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="H20" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="H21" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="H22" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="H23" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="H24" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="H25" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="H26" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="H27" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="H28" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="H29" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="H33" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="H34" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="H35" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="H36" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="H37" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="H38" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="H39" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="H40" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="H41" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="H42" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="H43" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
   </hyperlinks>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
update citation for MM systematic review paper
</commit_message>
<xml_diff>
--- a/_outputs.xlsx
+++ b/_outputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilro23p\Documents\rosswilson-nz.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A45A11-D672-4119-BFCA-64A8785FC944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA46AEE3-EE4E-4198-8A52-CFBCA1ACD474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="articles" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="482">
   <si>
     <t>authors</t>
   </si>
@@ -1494,6 +1494,9 @@
   </si>
   <si>
     <t>Musculoskeletal Science and Practice</t>
+  </si>
+  <si>
+    <t>10.1093/fampra/cmaf085</t>
   </si>
 </sst>
 </file>
@@ -1818,10 +1821,16 @@
         <v>20</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>13</v>
+        <v>249</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>133</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>14</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>481</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>474</v>

</xml_diff>

<commit_message>
update citation for GRoC validity paper
</commit_message>
<xml_diff>
--- a/_outputs.xlsx
+++ b/_outputs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilro23p\Documents\rosswilson-nz.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA46AEE3-EE4E-4198-8A52-CFBCA1ACD474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAC5E68B-B786-43EA-A6F4-82DB45E3541B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="484">
   <si>
     <t>authors</t>
   </si>
@@ -1497,6 +1497,12 @@
   </si>
   <si>
     <t>10.1093/fampra/cmaf085</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>103443</t>
   </si>
 </sst>
 </file>
@@ -1795,7 +1801,10 @@
         <v>480</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>13</v>
+        <v>482</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>483</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
add OA diagnoses medRxiv preprint
</commit_message>
<xml_diff>
--- a/_outputs.xlsx
+++ b/_outputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilro23p\Documents\rosswilson-nz.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAC5E68B-B786-43EA-A6F4-82DB45E3541B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F930C162-622B-49FA-9EE5-D3119D6A789C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="articles" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="489">
   <si>
     <t>authors</t>
   </si>
@@ -78,9 +78,6 @@
   </si>
   <si>
     <t>**Objective**&lt;br&gt;The aim of this study was to investigate the cost-effectiveness of low-dose colchicine prophylaxis for preventing gout flares when starting allopurinol using the “start-low go-slow” approach.&lt;br&gt;&lt;br&gt;**Methods**&lt;br&gt;Participants with gout, fulfilling the American College of Rheumatology recommendations for starting urate-lowering therapy and with serum urate ≥0.36 mmol/L (6mg/dL), were randomly allocated (1:1) to either colchicine (0.5 mg daily) or placebo for six months with a further six-month follow-up. All participants received allopurinol, with monthly increase in dose to achieve target urate &lt;0.36 mmol/L. The primary outcomes were incremental cost-effectiveness at 6-month and 1-year follow-up from the health system perspective, measured by incremental net monetary benefit (INMB) at a willingness-to-pay threshold equivalent to gross domestic product per capita.&lt;br&gt;&lt;br&gt;**Results**&lt;br&gt;Two hundred participants were randomized to either colchicine (n=100) or placebo (n=100). Mean costs were higher in the colchicine group over both 6 months and 1 year (adjusted mean difference $1 848 [95%CI −321 to 4 017] and $2 282 [95%CI −173 to 4 737], respectively). Quality-adjusted life years were slightly higher in the colchicine group over 6 months (adjusted mean difference 0.008 [95%CI −0.020 to 0.035]), but lower over 1 year (−0.015, [95%CI −0.039 to 0.010]). Treatment with colchicine was not found to be cost-effective at either 6-months or 12-months (INMB −$1 373 (95%CI −4 287 to 1 542) and −$3 191 (95%CI −6 274 to −107), probability of cost-effectiveness 17.7% and 1.5%, respectively). Similar results were obtained from a societal perspective.&lt;br&gt;&lt;br&gt;**Conclusion**&lt;br&gt;Six months of low-dose colchicine prophylaxis when starting allopurinol using the “start-low go-slow” approach is unlikely to be cost-effective over 12 months.</t>
-  </si>
-  <si>
-    <t>18 August 2025</t>
   </si>
   <si>
     <t>Pryymachenko Y, Wilson R, Abbott JH, Dowsey M, Choong P</t>
@@ -1504,12 +1501,30 @@
   <si>
     <t>103443</t>
   </si>
+  <si>
+    <t>25 November 2025</t>
+  </si>
+  <si>
+    <t>Osteoarthritis Diagnoses are Under-recorded in Primary Care Electronic Health Records in New Zealand</t>
+  </si>
+  <si>
+    <t>Rory Chistopherson, Yana Pryymachenko, Richelle Caya, Lívia Gaspar Fernandes, Yen Wei Lim, Moody Gayed, Andrés Pierobon, Tony Dowell, Ben Darlow, Jayden MacRae, and Haxby Abbott</t>
+  </si>
+  <si>
+    <t>medRxiv 2025.11.20.25340701</t>
+  </si>
+  <si>
+    <t>21 November 2025</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1101/2025.11.20.25340701</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1561,6 +1576,14 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1579,10 +1602,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1615,8 +1639,12 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1792,60 +1820,60 @@
     </row>
     <row r="2" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>475</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>476</v>
-      </c>
       <c r="C2" s="1" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>482</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>483</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>14</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>477</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>479</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="242.25" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>471</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>472</v>
-      </c>
       <c r="C3" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>14</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
@@ -1871,18 +1899,18 @@
         <v>16</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>17</v>
+        <v>483</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>20</v>
       </c>
       <c r="D5" s="1">
         <v>41</v>
@@ -1891,335 +1919,335 @@
         <v>6</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G5" s="1">
         <v>2024</v>
       </c>
       <c r="H5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="255" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="I6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="280.5" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H7" s="4" t="s">
+      <c r="I7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="89.25" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H8" s="4" t="s">
+      <c r="I8" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="J8" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="242.25" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H9" s="4" t="s">
+      <c r="I9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="G10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H10" s="4" t="s">
+      <c r="I10" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>70</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H11" s="4" t="s">
+      <c r="I11" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H12" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H12" s="4" t="s">
+      <c r="I12" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="293.25" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H13" s="4" t="s">
+      <c r="I13" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="165.75" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="D14" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="H14" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="I14" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="267.75" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="H15" s="4" t="s">
+      <c r="I15" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="280.5" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="5" t="s">
         <v>107</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>108</v>
       </c>
       <c r="D16" s="6">
         <v>52</v>
@@ -2228,853 +2256,853 @@
         <v>5</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G16" s="6">
         <v>2022</v>
       </c>
       <c r="H16" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="J16" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="J16" s="6" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="C17" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="D17" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="E17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H17" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="H17" s="10" t="s">
+      <c r="I17" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="J17" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="C18" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="D18" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="H18" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="I18" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="C19" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="D19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="H19" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="H19" s="10" t="s">
+      <c r="I19" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="J19" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="293.25" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="C20" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="D20" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F20" s="1" t="s">
+      <c r="G20" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="H20" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="G20" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="H20" s="10" t="s">
+      <c r="I20" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="I20" s="1" t="s">
+      <c r="J20" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="229.5" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="C21" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="D21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="H21" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="H21" s="10" t="s">
+      <c r="I21" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="J21" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="242.25" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="C22" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="C22" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F22" s="1" t="s">
+      <c r="G22" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H22" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="G22" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="H22" s="10" t="s">
+      <c r="I22" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="I22" s="1" t="s">
-        <v>157</v>
-      </c>
       <c r="J22" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="204" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B23" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="C23" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="C23" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="D23" s="1" t="s">
+      <c r="E23" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H23" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="H23" s="10" t="s">
+      <c r="I23" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="I23" s="1" t="s">
+      <c r="J23" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="153" x14ac:dyDescent="0.2">
       <c r="A24" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="C24" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="C24" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="E24" s="1" t="s">
+      <c r="F24" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H24" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="G24" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="H24" s="10" t="s">
+      <c r="I24" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="J24" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="191.25" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="B25" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="C25" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="D25" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F25" s="1" t="s">
+      <c r="G25" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H25" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="G25" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="H25" s="10" t="s">
+      <c r="I25" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="I25" s="1" t="s">
+      <c r="J25" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A26" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B26" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="C26" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="D26" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="E26" s="1" t="s">
+      <c r="F26" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="G26" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H26" s="10" t="s">
         <v>183</v>
       </c>
-      <c r="G26" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="H26" s="10" t="s">
+      <c r="I26" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="J26" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="153" x14ac:dyDescent="0.2">
       <c r="A27" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="B27" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="C27" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="D27" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="F27" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="G27" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H27" s="10" t="s">
         <v>191</v>
       </c>
-      <c r="G27" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="H27" s="10" t="s">
+      <c r="I27" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="I27" s="1" t="s">
+      <c r="J27" s="1" t="s">
         <v>193</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="191.25" x14ac:dyDescent="0.2">
       <c r="A28" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="B28" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="C28" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="D28" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="E28" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="F28" s="1" t="s">
+      <c r="G28" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H28" s="10" t="s">
         <v>199</v>
       </c>
-      <c r="G28" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="H28" s="10" t="s">
+      <c r="I28" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="I28" s="1" t="s">
+      <c r="J28" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="191.25" x14ac:dyDescent="0.2">
       <c r="A29" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="B29" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="C29" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="C29" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="F29" s="1" t="s">
+      <c r="G29" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H29" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="G29" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="H29" s="10" t="s">
+      <c r="I29" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="I29" s="1" t="s">
+      <c r="J29" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="102" x14ac:dyDescent="0.2">
       <c r="A30" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="B30" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="C30" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="D30" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="E30" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="F30" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G30" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="I30" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="G30" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="I30" s="1" t="s">
-        <v>215</v>
-      </c>
       <c r="J30" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="165.75" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="B31" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="C31" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="D31" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="G31" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="G31" s="1" t="s">
+      <c r="I31" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="I31" s="1" t="s">
+      <c r="J31" s="1" t="s">
         <v>223</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="165.75" x14ac:dyDescent="0.2">
       <c r="A32" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="B32" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="C32" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="C32" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="E32" s="1" t="s">
+      <c r="F32" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="G32" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="I32" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="G32" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="I32" s="1" t="s">
+      <c r="J32" s="1" t="s">
         <v>229</v>
-      </c>
-      <c r="J32" s="1" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A33" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="B33" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="C33" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="D33" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="E33" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="E33" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="F33" s="1" t="s">
+      <c r="G33" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="H33" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="G33" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="H33" s="10" t="s">
+      <c r="I33" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="I33" s="1" t="s">
+      <c r="J33" s="1" t="s">
         <v>237</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="242.25" x14ac:dyDescent="0.2">
       <c r="A34" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="B34" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="C34" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="C34" s="9" t="s">
+      <c r="D34" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="E34" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="E34" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F34" s="1" t="s">
+      <c r="G34" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="H34" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="G34" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="H34" s="10" t="s">
+      <c r="I34" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="I34" s="1" t="s">
+      <c r="J34" s="1" t="s">
         <v>245</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="178.5" x14ac:dyDescent="0.2">
       <c r="A35" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B35" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C35" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="D35" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="E35" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F35" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="E35" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F35" s="1" t="s">
+      <c r="G35" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="G35" s="1" t="s">
+      <c r="H35" s="10" t="s">
         <v>251</v>
       </c>
-      <c r="H35" s="10" t="s">
+      <c r="I35" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="I35" s="1" t="s">
+      <c r="J35" s="1" t="s">
         <v>253</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A36" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B36" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="C36" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="D36" s="1" t="s">
+      <c r="E36" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F36" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="E36" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F36" s="1" t="s">
+      <c r="G36" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="H36" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="G36" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="H36" s="10" t="s">
+      <c r="I36" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="I36" s="1" t="s">
+      <c r="J36" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A37" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="B37" s="8" t="s">
         <v>261</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="C37" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="D37" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="E37" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="E37" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="H37" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="G37" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="H37" s="10" t="s">
+      <c r="I37" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="J37" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A38" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="B38" s="8" t="s">
         <v>269</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="C38" s="9" t="s">
         <v>270</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="D38" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="D38" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F38" s="1" t="s">
+      <c r="G38" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="G38" s="1" t="s">
+      <c r="H38" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="H38" s="10" t="s">
+      <c r="I38" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="I38" s="1" t="s">
+      <c r="J38" s="1" t="s">
         <v>275</v>
-      </c>
-      <c r="J38" s="1" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="255" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B39" s="8" t="s">
         <v>277</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="C39" s="9" t="s">
         <v>278</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="D39" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="F39" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="G39" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="G39" s="1" t="s">
+      <c r="H39" s="10" t="s">
         <v>282</v>
       </c>
-      <c r="H39" s="10" t="s">
+      <c r="I39" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="I39" s="1" t="s">
+      <c r="J39" s="1" t="s">
         <v>284</v>
-      </c>
-      <c r="J39" s="1" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="267.75" x14ac:dyDescent="0.2">
       <c r="A40" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B40" s="8" t="s">
         <v>286</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="C40" s="9" t="s">
         <v>287</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="D40" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G40" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="D40" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G40" s="1" t="s">
+      <c r="H40" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="H40" s="10" t="s">
+      <c r="I40" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="I40" s="1" t="s">
+      <c r="J40" s="1" t="s">
         <v>291</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="216.75" x14ac:dyDescent="0.2">
       <c r="A41" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="B41" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="C41" s="9" t="s">
         <v>294</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="D41" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="F41" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="G41" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="G41" s="1" t="s">
+      <c r="H41" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="H41" s="10" t="s">
+      <c r="I41" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="I41" s="1" t="s">
+      <c r="J41" s="1" t="s">
         <v>300</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="382.5" x14ac:dyDescent="0.2">
       <c r="A42" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="B42" s="8" t="s">
         <v>302</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="C42" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="D42" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="D42" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F42" s="1" t="s">
+      <c r="G42" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="G42" s="1" t="s">
+      <c r="H42" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="H42" s="10" t="s">
+      <c r="I42" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="I42" s="1" t="s">
+      <c r="J42" s="1" t="s">
         <v>308</v>
-      </c>
-      <c r="J42" s="1" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="165.75" x14ac:dyDescent="0.2">
       <c r="A43" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B43" s="8" t="s">
         <v>310</v>
       </c>
-      <c r="B43" s="8" t="s">
+      <c r="C43" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="C43" s="9" t="s">
-        <v>288</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F43" s="1" t="s">
+      <c r="G43" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="H43" s="10" t="s">
         <v>312</v>
       </c>
-      <c r="G43" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="H43" s="10" t="s">
+      <c r="I43" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="I43" s="1" t="s">
+      <c r="J43" s="1" t="s">
         <v>314</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>315</v>
       </c>
     </row>
   </sheetData>
@@ -3139,10 +3167,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>316</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>317</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>9</v>
@@ -3151,540 +3179,540 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="8" t="s">
         <v>321</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="E2" s="1" t="s">
         <v>322</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="8" t="s">
         <v>326</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
+        <v>327</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="8" t="s">
         <v>330</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="5" spans="1:5" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="8" t="s">
         <v>334</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>335</v>
       </c>
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>338</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="8" t="s">
         <v>342</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>344</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>346</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>348</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
+        <v>349</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>350</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
+        <v>351</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>333</v>
-      </c>
-      <c r="C12" s="1" t="s">
+      <c r="D12" s="8" t="s">
         <v>353</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>354</v>
-      </c>
       <c r="E12" s="1" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>358</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>357</v>
-      </c>
       <c r="D14" s="9" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>357</v>
-      </c>
       <c r="D15" s="9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>361</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>363</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="C17" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="D17" s="9" t="s">
         <v>365</v>
       </c>
-      <c r="D17" s="9" t="s">
-        <v>366</v>
-      </c>
       <c r="E17" s="1" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>367</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>368</v>
-      </c>
       <c r="E18" s="8" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
+        <v>369</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>333</v>
-      </c>
-      <c r="C20" s="1" t="s">
+      <c r="D20" s="9" t="s">
         <v>371</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>373</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="C21" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>374</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>371</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>376</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="C22" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="D22" s="9" t="s">
         <v>378</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>324</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>325</v>
-      </c>
-      <c r="C23" s="1" t="s">
+      <c r="D23" s="9" t="s">
         <v>381</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A24" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>324</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="B24" s="8" t="s">
-        <v>325</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>381</v>
-      </c>
       <c r="D24" s="9" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
+        <v>383</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>333</v>
-      </c>
-      <c r="C25" s="1" t="s">
+      <c r="D25" s="9" t="s">
         <v>385</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A26" s="8" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="D26" s="9" t="s">
         <v>385</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A27" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>377</v>
-      </c>
       <c r="C27" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="D27" s="9" t="s">
         <v>385</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="D28" s="9" t="s">
         <v>388</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>385</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>389</v>
-      </c>
       <c r="E28" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
+        <v>391</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>377</v>
-      </c>
-      <c r="C31" s="1" t="s">
+      <c r="D31" s="9" t="s">
         <v>393</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="89.25" x14ac:dyDescent="0.2">
       <c r="A32" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="C32" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="D32" s="9" t="s">
         <v>397</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A33" s="8" t="s">
+        <v>398</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>356</v>
-      </c>
-      <c r="C33" s="1" t="s">
+      <c r="D33" s="9" t="s">
         <v>400</v>
       </c>
-      <c r="D33" s="9" t="s">
-        <v>401</v>
-      </c>
       <c r="E33" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A34" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="C34" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="D34" s="9" t="s">
         <v>404</v>
       </c>
-      <c r="D34" s="9" t="s">
-        <v>405</v>
-      </c>
       <c r="E34" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A35" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>377</v>
-      </c>
       <c r="C35" s="1" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B36" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="D36" s="9" t="s">
         <v>408</v>
       </c>
-      <c r="D36" s="9" t="s">
-        <v>409</v>
-      </c>
       <c r="E36" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>
@@ -3699,7 +3727,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="101.42578125" style="1" customWidth="1"/>
@@ -3715,243 +3743,261 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>412</v>
+        <v>410</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>484</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>413</v>
+        <v>485</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>486</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>415</v>
+        <v>487</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E4" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="E3" s="2" t="s">
+    </row>
+    <row r="5" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
         <v>419</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
+      <c r="B5" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E5" s="7" t="s">
         <v>422</v>
       </c>
-      <c r="E4" s="7" t="s">
+    </row>
+    <row r="6" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
         <v>423</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
+      <c r="B6" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E6" s="7" t="s">
         <v>426</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
-        <v>428</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>429</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>431</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E8" s="7" t="s">
         <v>434</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
-        <v>436</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>437</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>438</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
+        <v>443</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>440</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>441</v>
-      </c>
-      <c r="D11" s="1" t="s">
+      <c r="E12" s="10" t="s">
         <v>449</v>
       </c>
-      <c r="E11" s="10" t="s">
+    </row>
+    <row r="13" spans="1:5" ht="306" x14ac:dyDescent="0.2">
+      <c r="A13" s="9" t="s">
         <v>450</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="306" x14ac:dyDescent="0.2">
-      <c r="A12" s="9" t="s">
+      <c r="B13" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="C13" s="8" t="s">
         <v>452</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="D13" s="8" t="s">
         <v>453</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="E13" s="10" t="s">
         <v>454</v>
       </c>
-      <c r="E12" s="10" t="s">
+    </row>
+    <row r="14" spans="1:5" ht="280.5" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="280.5" x14ac:dyDescent="0.2">
-      <c r="A13" s="9" t="s">
+      <c r="C14" s="8" t="s">
         <v>456</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="D14" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E14" s="10" t="s">
         <v>458</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A14" s="9" t="s">
-        <v>460</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>461</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>462</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
-        <v>464</v>
+        <v>459</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>466</v>
+        <v>461</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>467</v>
+        <v>462</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
+        <v>463</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>464</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>465</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A17" s="9" t="s">
+        <v>467</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>468</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="C17" s="8" t="s">
+        <v>465</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>469</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>466</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>470</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E4" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
-    <hyperlink ref="E5" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
-    <hyperlink ref="E6" r:id="rId3" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
-    <hyperlink ref="E7" r:id="rId4" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
-    <hyperlink ref="E8" r:id="rId5" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
-    <hyperlink ref="E9" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
-    <hyperlink ref="E10" r:id="rId7" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
-    <hyperlink ref="E11" r:id="rId8" xr:uid="{00000000-0004-0000-0200-000007000000}"/>
-    <hyperlink ref="E12" r:id="rId9" xr:uid="{00000000-0004-0000-0200-000008000000}"/>
-    <hyperlink ref="E13" r:id="rId10" xr:uid="{00000000-0004-0000-0200-000009000000}"/>
+    <hyperlink ref="E5" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="E6" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
+    <hyperlink ref="E7" r:id="rId3" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
+    <hyperlink ref="E8" r:id="rId4" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
+    <hyperlink ref="E9" r:id="rId5" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
+    <hyperlink ref="E10" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
+    <hyperlink ref="E11" r:id="rId7" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
+    <hyperlink ref="E12" r:id="rId8" xr:uid="{00000000-0004-0000-0200-000007000000}"/>
+    <hyperlink ref="E13" r:id="rId9" xr:uid="{00000000-0004-0000-0200-000008000000}"/>
+    <hyperlink ref="E14" r:id="rId10" xr:uid="{00000000-0004-0000-0200-000009000000}"/>
+    <hyperlink ref="E2" r:id="rId11" xr:uid="{6D944E76-FFB2-4EFB-BB13-F5F081889010}"/>
   </hyperlinks>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
add IDI symposium presentation
</commit_message>
<xml_diff>
--- a/_outputs.xlsx
+++ b/_outputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilro23p\Documents\rosswilson-nz.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F930C162-622B-49FA-9EE5-D3119D6A789C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53199F98-4CBF-47B2-BCF1-D579027906D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="articles" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="492">
   <si>
     <t>authors</t>
   </si>
@@ -1518,6 +1518,15 @@
   </si>
   <si>
     <t>https://doi.org/10.1101/2025.11.20.25340701</t>
+  </si>
+  <si>
+    <t>University of Otago Research Symposium: Harnessing Linked Population-Level Data for Health Research</t>
+  </si>
+  <si>
+    <t>November 2025</t>
+  </si>
+  <si>
+    <t>Osteoarthritis diagnoses are under-recorded in primary care electronic health records in New Zealand</t>
   </si>
 </sst>
 </file>
@@ -3154,7 +3163,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.5703125" style="1" customWidth="1"/>
@@ -3182,100 +3191,103 @@
         <v>317</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>318</v>
+        <v>489</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>319</v>
+        <v>332</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>321</v>
+        <v>490</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>491</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
+    <row r="3" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
         <v>323</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D4" s="8" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="41.25" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
+    <row r="5" spans="1:5" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A5" s="11" t="s">
         <v>327</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D5" s="8" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="5" spans="1:5" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A5" s="8" t="s">
+    <row r="6" spans="1:5" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A6" s="8" t="s">
         <v>331</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D6" s="8" t="s">
         <v>334</v>
       </c>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>338</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A7" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>340</v>
@@ -3284,12 +3296,12 @@
         <v>341</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="76.5" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>340</v>
@@ -3298,12 +3310,12 @@
         <v>341</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>340</v>
@@ -3312,12 +3324,12 @@
         <v>341</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>340</v>
@@ -3326,57 +3338,54 @@
         <v>341</v>
       </c>
       <c r="D11" s="8" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A12" s="8" t="s">
+        <v>349</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A12" s="8" t="s">
+    <row r="13" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A13" s="8" t="s">
         <v>351</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D13" s="8" t="s">
         <v>353</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>355</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>356</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="2" t="s">
         <v>355</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="D14" s="9" t="s">
-        <v>358</v>
-      </c>
-      <c r="E14" s="1" t="s">
+      <c r="D14" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>338</v>
       </c>
     </row>
@@ -3391,57 +3400,57 @@
         <v>356</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A17" s="11" t="s">
         <v>323</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B17" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D17" s="9" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="63.75" x14ac:dyDescent="0.2">
-      <c r="A17" s="8" t="s">
+    <row r="18" spans="1:5" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A18" s="8" t="s">
         <v>362</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B18" s="8" t="s">
         <v>363</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D18" s="9" t="s">
         <v>365</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A18" s="11" t="s">
-        <v>323</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>366</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>367</v>
-      </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="1" t="s">
         <v>322</v>
       </c>
     </row>
@@ -3456,63 +3465,66 @@
         <v>366</v>
       </c>
       <c r="D19" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A20" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="D20" s="9" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="63.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="8" t="s">
+    <row r="21" spans="1:5" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="8" t="s">
         <v>369</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>332</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A21" s="8" t="s">
-        <v>372</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>373</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>370</v>
       </c>
       <c r="D21" s="9" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A22" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="D22" s="9" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="8" t="s">
+    <row r="23" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A23" s="8" t="s">
         <v>375</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B23" s="8" t="s">
         <v>376</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C23" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D23" s="9" t="s">
         <v>378</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A23" s="8" t="s">
-        <v>379</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>324</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>380</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="76.5" x14ac:dyDescent="0.2">
@@ -3526,29 +3538,29 @@
         <v>380</v>
       </c>
       <c r="D24" s="9" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A25" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>324</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>382</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A25" s="8" t="s">
-        <v>383</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>332</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A26" s="8" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>384</v>
@@ -3559,10 +3571,10 @@
     </row>
     <row r="27" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A27" s="8" t="s">
-        <v>375</v>
+        <v>386</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>376</v>
+        <v>340</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>384</v>
@@ -3571,25 +3583,22 @@
         <v>385</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A28" s="8" t="s">
-        <v>354</v>
+        <v>375</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>387</v>
+        <v>376</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>384</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>388</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>338</v>
+        <v>385</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="1" t="s">
+      <c r="A29" s="8" t="s">
         <v>354</v>
       </c>
       <c r="B29" s="1" t="s">
@@ -3599,7 +3608,7 @@
         <v>384</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>338</v>
@@ -3616,69 +3625,69 @@
         <v>384</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A31" s="8" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>390</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A32" s="8" t="s">
         <v>391</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B32" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C32" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="D31" s="9" t="s">
+      <c r="D32" s="9" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="89.25" x14ac:dyDescent="0.2">
-      <c r="A32" s="8" t="s">
+    <row r="33" spans="1:5" ht="89.25" x14ac:dyDescent="0.2">
+      <c r="A33" s="8" t="s">
         <v>394</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B33" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C33" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="D33" s="9" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A33" s="8" t="s">
+    <row r="34" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A34" s="8" t="s">
         <v>398</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C34" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="D34" s="9" t="s">
         <v>400</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A34" s="8" t="s">
-        <v>401</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>402</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="D34" s="9" t="s">
-        <v>404</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>338</v>
@@ -3686,32 +3695,49 @@
     </row>
     <row r="35" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A35" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A36" s="8" t="s">
         <v>375</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B36" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C36" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="D35" s="9" t="s">
+      <c r="D36" s="9" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B37" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C37" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="D37" s="9" t="s">
         <v>408</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="E37" s="1" t="s">
         <v>338</v>
       </c>
     </row>

</xml_diff>